<commit_message>
Improve fixed-layout video plan handoff
</commit_message>
<xml_diff>
--- a/docs/templates/manual-video-handoff.xlsx
+++ b/docs/templates/manual-video-handoff.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频方案" sheetId="1" r:id="R7a4e9f18ec994104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频方案" sheetId="1" r:id="R9284c7b3069943f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参考资产" sheetId="2" r:id="Rf7d481968167435e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32,6 +33,29 @@
     </x:font>
     <x:font>
       <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF23312E"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF26433C"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
       <x:sz val="10"/>
       <x:color rgb="FF23312E"/>
       <x:name val="Aptos"/>
@@ -39,12 +63,6 @@
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF23312E"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
@@ -70,23 +88,6 @@
       <x:color rgb="FF23312E"/>
       <x:name val="Aptos"/>
     </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF23312E"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF26433C"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="12"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Aptos"/>
-    </x:font>
   </x:fonts>
   <x:fills count="9">
     <x:fill>
@@ -94,16 +95,6 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE8DED0"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFDFC"/>
-      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -122,6 +113,11 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFDFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
         <x:fgColor rgb="FFDDE8E0"/>
       </x:patternFill>
     </x:fill>
@@ -130,13 +126,56 @@
         <x:fgColor rgb="FFF4EEE6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8DED0"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="8">
+  <x:borders count="10">
     <x:border>
       <x:left/>
       <x:right/>
       <x:top/>
       <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="medium">
+        <x:color rgb="FFA8693B"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE9E2D8"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFE9E2D8"/>
+      </x:right>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE9E2D8"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFD6CDC1"/>
+      </x:bottom>
       <x:diagonal/>
     </x:border>
     <x:border>
@@ -150,10 +189,12 @@
     </x:border>
     <x:border>
       <x:left/>
-      <x:right/>
+      <x:right style="thin">
+        <x:color rgb="FFE9E2D8"/>
+      </x:right>
       <x:top/>
-      <x:bottom style="medium">
-        <x:color rgb="FFA8693B"/>
+      <x:bottom style="thin">
+        <x:color rgb="FFD6CDC1"/>
       </x:bottom>
       <x:diagonal/>
     </x:border>
@@ -190,33 +231,11 @@
       </x:bottom>
       <x:diagonal/>
     </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFE9E2D8"/>
-      </x:left>
-      <x:right/>
-      <x:top/>
-      <x:bottom style="thin">
-        <x:color rgb="FFD6CDC1"/>
-      </x:bottom>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right style="thin">
-        <x:color rgb="FFE9E2D8"/>
-      </x:right>
-      <x:top/>
-      <x:bottom style="thin">
-        <x:color rgb="FFD6CDC1"/>
-      </x:bottom>
-      <x:diagonal/>
-    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="57">
+  <x:cellXfs count="75">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -234,128 +253,178 @@
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="11" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -604,290 +673,301 @@
       <x:c r="J2" s="4"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="35"/>
-      <x:c r="B3" s="35"/>
-      <x:c r="C3" s="35"/>
-      <x:c r="D3" s="35"/>
-      <x:c r="E3" s="35"/>
-      <x:c r="F3" s="35"/>
-      <x:c r="G3" s="35"/>
-      <x:c r="H3" s="35"/>
-      <x:c r="I3" s="35"/>
-      <x:c r="J3" s="35"/>
+      <x:c r="A3" s="14"/>
+      <x:c r="B3" s="14"/>
+      <x:c r="C3" s="14"/>
+      <x:c r="D3" s="14"/>
+      <x:c r="E3" s="14"/>
+      <x:c r="F3" s="14"/>
+      <x:c r="G3" s="14"/>
+      <x:c r="H3" s="14"/>
+      <x:c r="I3" s="14"/>
+      <x:c r="J3" s="14"/>
     </x:row>
     <x:row r="4" ht="21" customHeight="1">
-      <x:c r="A4" s="36" t="str">
+      <x:c r="A4" s="61" t="str">
         <x:v>作品名</x:v>
       </x:c>
-      <x:c r="B4" s="36" t="str"/>
-      <x:c r="C4" s="36" t="str">
+      <x:c r="B4" s="61" t="str"/>
+      <x:c r="C4" s="61" t="str">
         <x:v>产品 / 主体</x:v>
       </x:c>
-      <x:c r="D4" s="36" t="str"/>
-      <x:c r="E4" s="36" t="str">
+      <x:c r="D4" s="61" t="str"/>
+      <x:c r="E4" s="61" t="str">
         <x:v>受众</x:v>
       </x:c>
-      <x:c r="F4" s="36" t="str"/>
-      <x:c r="G4" s="36" t="str">
+      <x:c r="F4" s="61" t="str"/>
+      <x:c r="G4" s="61" t="str">
         <x:v>画幅</x:v>
       </x:c>
-      <x:c r="H4" s="36" t="str"/>
-      <x:c r="I4" s="36" t="str">
+      <x:c r="H4" s="61" t="str"/>
+      <x:c r="I4" s="61" t="str">
         <x:v>总时长</x:v>
       </x:c>
-      <x:c r="J4" s="36" t="str"/>
+      <x:c r="J4" s="61" t="str"/>
     </x:row>
     <x:row r="5" ht="21" customHeight="1">
-      <x:c r="A5" s="37" t="str"/>
-      <x:c r="B5" s="37" t="str"/>
-      <x:c r="C5" s="37" t="str"/>
-      <x:c r="D5" s="37" t="str"/>
-      <x:c r="E5" s="37" t="str"/>
-      <x:c r="F5" s="37" t="str"/>
-      <x:c r="G5" s="37" t="str"/>
-      <x:c r="H5" s="37" t="str"/>
-      <x:c r="I5" s="37" t="str"/>
-      <x:c r="J5" s="37" t="str"/>
+      <x:c r="A5" s="62" t="str"/>
+      <x:c r="B5" s="62" t="str"/>
+      <x:c r="C5" s="62" t="str"/>
+      <x:c r="D5" s="62" t="str"/>
+      <x:c r="E5" s="62" t="str"/>
+      <x:c r="F5" s="62" t="str"/>
+      <x:c r="G5" s="62" t="str"/>
+      <x:c r="H5" s="62" t="str"/>
+      <x:c r="I5" s="62" t="str"/>
+      <x:c r="J5" s="62" t="str"/>
     </x:row>
     <x:row r="6" ht="21" customHeight="1">
-      <x:c r="A6" s="36" t="str">
+      <x:c r="A6" s="61" t="str">
         <x:v>声音方向</x:v>
       </x:c>
-      <x:c r="B6" s="36" t="str"/>
-      <x:c r="C6" s="36" t="str">
+      <x:c r="B6" s="61" t="str"/>
+      <x:c r="C6" s="61" t="str">
         <x:v>整体调性</x:v>
       </x:c>
-      <x:c r="D6" s="36" t="str"/>
-      <x:c r="E6" s="36" t="str">
+      <x:c r="D6" s="61" t="str"/>
+      <x:c r="E6" s="61" t="str">
         <x:v>核心信息</x:v>
       </x:c>
-      <x:c r="F6" s="36" t="str"/>
-      <x:c r="G6" s="36" t="str">
+      <x:c r="F6" s="61" t="str"/>
+      <x:c r="G6" s="61" t="str">
         <x:v>交付日期</x:v>
       </x:c>
-      <x:c r="H6" s="36" t="str"/>
-      <x:c r="I6" s="36" t="str">
+      <x:c r="H6" s="61" t="str"/>
+      <x:c r="I6" s="61" t="str">
         <x:v>方案版本</x:v>
       </x:c>
-      <x:c r="J6" s="36" t="str"/>
+      <x:c r="J6" s="61" t="str"/>
     </x:row>
     <x:row r="7" ht="21" customHeight="1">
-      <x:c r="A7" s="37" t="str"/>
-      <x:c r="B7" s="37" t="str"/>
-      <x:c r="C7" s="37" t="str"/>
-      <x:c r="D7" s="37" t="str"/>
-      <x:c r="E7" s="37" t="str"/>
-      <x:c r="F7" s="37" t="str"/>
-      <x:c r="G7" s="37" t="str"/>
-      <x:c r="H7" s="37" t="str"/>
-      <x:c r="I7" s="37" t="str"/>
-      <x:c r="J7" s="37" t="str"/>
+      <x:c r="A7" s="62" t="str"/>
+      <x:c r="B7" s="62" t="str"/>
+      <x:c r="C7" s="62" t="str"/>
+      <x:c r="D7" s="62" t="str"/>
+      <x:c r="E7" s="62" t="str"/>
+      <x:c r="F7" s="62" t="str"/>
+      <x:c r="G7" s="62" t="str"/>
+      <x:c r="H7" s="62" t="str"/>
+      <x:c r="I7" s="62" t="str"/>
+      <x:c r="J7" s="62" t="str"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="35"/>
-      <x:c r="B8" s="35"/>
-      <x:c r="C8" s="35"/>
-      <x:c r="D8" s="35"/>
-      <x:c r="E8" s="35"/>
-      <x:c r="F8" s="35"/>
-      <x:c r="G8" s="35"/>
-      <x:c r="H8" s="35"/>
-      <x:c r="I8" s="35"/>
-      <x:c r="J8" s="35"/>
+      <x:c r="A8" s="14"/>
+      <x:c r="B8" s="14"/>
+      <x:c r="C8" s="14"/>
+      <x:c r="D8" s="14"/>
+      <x:c r="E8" s="14"/>
+      <x:c r="F8" s="14"/>
+      <x:c r="G8" s="14"/>
+      <x:c r="H8" s="14"/>
+      <x:c r="I8" s="14"/>
+      <x:c r="J8" s="14"/>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="53" t="str">
+      <x:c r="A9" s="7" t="str">
         <x:v>生成片段清单</x:v>
       </x:c>
-      <x:c r="B9" s="53"/>
-      <x:c r="C9" s="53"/>
-      <x:c r="D9" s="53"/>
-      <x:c r="E9" s="53"/>
-      <x:c r="F9" s="53"/>
-      <x:c r="G9" s="53"/>
-      <x:c r="H9" s="53"/>
-      <x:c r="I9" s="53"/>
-      <x:c r="J9" s="53"/>
+      <x:c r="B9" s="7"/>
+      <x:c r="C9" s="7"/>
+      <x:c r="D9" s="7"/>
+      <x:c r="E9" s="7"/>
+      <x:c r="F9" s="7"/>
+      <x:c r="G9" s="7"/>
+      <x:c r="H9" s="7"/>
+      <x:c r="I9" s="7"/>
+      <x:c r="J9" s="7"/>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="54" t="str">
+      <x:c r="A10" s="73" t="str">
         <x:v>片段</x:v>
       </x:c>
-      <x:c r="B10" s="55" t="str">
+      <x:c r="B10" s="13" t="str">
         <x:v>整片位置
 建议时长</x:v>
       </x:c>
-      <x:c r="C10" s="55" t="str">
+      <x:c r="C10" s="13" t="str">
         <x:v>关联分镜 / 段内节奏</x:v>
       </x:c>
-      <x:c r="D10" s="55" t="str">
+      <x:c r="D10" s="13" t="str">
         <x:v>场景、画面与动作</x:v>
       </x:c>
-      <x:c r="E10" s="55" t="str">
-        <x:v>参考图组</x:v>
-      </x:c>
-      <x:c r="F10" s="55" t="str">
+      <x:c r="E10" s="13" t="str">
+        <x:v>角色 / 场景 / 产品参考</x:v>
+      </x:c>
+      <x:c r="F10" s="13" t="str">
         <x:v>口播 / 对白全文</x:v>
       </x:c>
-      <x:c r="G10" s="55" t="str">
+      <x:c r="G10" s="13" t="str">
         <x:v>屏幕文字</x:v>
       </x:c>
-      <x:c r="H10" s="55" t="str">
+      <x:c r="H10" s="13" t="str">
         <x:v>完整生成提示词</x:v>
       </x:c>
-      <x:c r="I10" s="55" t="str">
+      <x:c r="I10" s="13" t="str">
         <x:v>前后衔接</x:v>
       </x:c>
-      <x:c r="J10" s="56" t="str">
+      <x:c r="J10" s="74" t="str">
         <x:v>验收要点</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="220" customHeight="1">
-      <x:c r="A11" s="49" t="str">
+    <x:row r="11" ht="250" customHeight="1">
+      <x:c r="A11" s="71" t="str">
         <x:v>片段 01
 模板示意</x:v>
       </x:c>
-      <x:c r="B11" s="40" t="str">
+      <x:c r="B11" s="65" t="str">
         <x:v>00:00–00:10
 建议 10 秒
 9:16</x:v>
       </x:c>
-      <x:c r="C11" s="40" t="str">
+      <x:c r="C11" s="65" t="str">
         <x:v>对应原分镜 01–03（示意）
 0–3 秒：人物注意到杯子
 3–7 秒：拿起并打开杯盖
 7–10 秒：自然饮用</x:v>
       </x:c>
-      <x:c r="D11" s="40" t="str">
+      <x:c r="D11" s="65" t="str">
         <x:v>暖色窗边桌面。一位人物坐在桌边，视线先落在杯子上，拿起杯子，顺手打开杯盖并喝一口。动作连贯，自然停顿。</x:v>
       </x:c>
-      <x:c r="E11" s="44" t="str">
-        <x:v>在此嵌入实际参考图
-人物：桌边人物
-产品：杯子
-场景：暖色窗边
-占位仅示意，交付时替换为真实生成图片。</x:v>
-      </x:c>
-      <x:c r="F11" s="40" t="str">
+      <x:c r="E11" s="27" t="str">
+        <x:v>本段图 1：P01 产品参考
+产品外形、材质与标志
+本段图 2：R01 角色参考
+角色身份与造型
+本段图 3：S01 场景参考
+窗边布局、光线与陈设
+按本段实际需要增减；实际交付时将对应真图嵌入本单元格。</x:v>
+      </x:c>
+      <x:c r="F11" s="65" t="str">
         <x:v>画外音（后期配音）：
 “忙碌的间隙，也该有一口舒服的热咖啡。”</x:v>
       </x:c>
-      <x:c r="G11" s="40" t="str">
+      <x:c r="G11" s="65" t="str">
         <x:v>留给自己
 十秒热度</x:v>
       </x:c>
-      <x:c r="H11" s="46" t="str">
-        <x:v>竖屏，暖色自然晨光。桌边人物坐在窗旁，画面中保持同一只简洁咖啡杯。她不现场发声，先看向杯子，再自然地拿起杯子，打开杯盖，停顿片刻后喝一口。镜头从中景缓慢推进到半身近景，人物动作连贯，杯型与画面氛围稳定。后期画外音逐字使用“忙碌的间隙，也该有一口舒服的热咖啡。”；屏幕文字后期添加，画面中不生成文字。</x:v>
-      </x:c>
-      <x:c r="I11" s="40" t="str">
+      <x:c r="H11" s="68" t="str">
+        <x:v>参考图按本段图序使用：图 1 为 P01，保持产品外形、材质与标志；图 2 为 R01，保持角色身份与造型；图 3 为 S01，保持窗边布局、暖色光线与陈设。竖屏，暖色自然晨光。角色坐在窗旁，不现场发声，先看向产品，再自然地拿起产品，完成打开与饮用动作。镜头从中景缓慢推进到半身近景，动作连贯，主体与空间关系稳定。后期画外音逐字使用“忙碌的间隙，也该有一口舒服的热咖啡。”；屏幕文字后期添加，画面中不生成文字。</x:v>
+      </x:c>
+      <x:c r="I11" s="65" t="str">
         <x:v>承接：上一片段已建立窗边桌面与杯子。
 下一片段：人物饮用后轻松微笑，转向产品细节。</x:v>
       </x:c>
-      <x:c r="J11" s="50" t="str">
+      <x:c r="J11" s="72" t="str">
         <x:v>人物、杯型、窗边光线稳定。
 拿杯、开盖、饮用三步连贯。
 后期画外音与口播列逐字一致。</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="142" customHeight="1">
-      <x:c r="A12" s="51" t="str">
+    <x:row r="12" ht="158" customHeight="1">
+      <x:c r="A12" s="32" t="str">
         <x:v>片段 02</x:v>
       </x:c>
-      <x:c r="B12" s="41" t="str">
+      <x:c r="B12" s="26" t="str">
         <x:v>填写整片位置、时长与画幅</x:v>
       </x:c>
-      <x:c r="C12" s="41" t="str">
+      <x:c r="C12" s="26" t="str">
         <x:v>填写关联分镜编号与段内节奏
 不要拆成独立生成任务</x:v>
       </x:c>
-      <x:c r="D12" s="41" t="str">
+      <x:c r="D12" s="26" t="str">
         <x:v>填写场景、构图、人物与动作</x:v>
       </x:c>
-      <x:c r="E12" s="44" t="str">
-        <x:v>在此嵌入实际参考图
-注明人物 / 产品 / 场景用途</x:v>
-      </x:c>
-      <x:c r="F12" s="41" t="str">
+      <x:c r="E12" s="27" t="str">
+        <x:v>填写本段图序与图 ID
+如图 1：P__ 产品参考
+图 2：R__ 角色参考
+图 3：S__ 场景参考
+按需增减，并嵌入对应真图</x:v>
+      </x:c>
+      <x:c r="F12" s="26" t="str">
         <x:v>填写口播或对白全文</x:v>
       </x:c>
-      <x:c r="G12" s="41" t="str">
+      <x:c r="G12" s="26" t="str">
         <x:v>填写屏幕文字</x:v>
       </x:c>
-      <x:c r="H12" s="46" t="str">
+      <x:c r="H12" s="68" t="str">
         <x:v>填写一次生成可直接复制的完整提示词</x:v>
       </x:c>
-      <x:c r="I12" s="41" t="str">
+      <x:c r="I12" s="26" t="str">
         <x:v>填写与前后片段的衔接</x:v>
       </x:c>
-      <x:c r="J12" s="52" t="str">
+      <x:c r="J12" s="29" t="str">
         <x:v>填写需核对的画面与动作要点</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="142" customHeight="1">
-      <x:c r="A13" s="49" t="str">
+    <x:row r="13" ht="158" customHeight="1">
+      <x:c r="A13" s="71" t="str">
         <x:v>片段 03</x:v>
       </x:c>
-      <x:c r="B13" s="40" t="str">
+      <x:c r="B13" s="65" t="str">
         <x:v>填写整片位置、时长与画幅</x:v>
       </x:c>
-      <x:c r="C13" s="40" t="str">
+      <x:c r="C13" s="65" t="str">
         <x:v>填写关联分镜编号与段内节奏
 不要拆成独立生成任务</x:v>
       </x:c>
-      <x:c r="D13" s="40" t="str">
+      <x:c r="D13" s="65" t="str">
         <x:v>填写场景、构图、人物与动作</x:v>
       </x:c>
-      <x:c r="E13" s="44" t="str">
-        <x:v>在此嵌入实际参考图
-注明人物 / 产品 / 场景用途</x:v>
-      </x:c>
-      <x:c r="F13" s="40" t="str">
+      <x:c r="E13" s="27" t="str">
+        <x:v>填写本段图序与图 ID
+如图 1：P__ 产品参考
+图 2：R__ 角色参考
+图 3：S__ 场景参考
+按需增减，并嵌入对应真图</x:v>
+      </x:c>
+      <x:c r="F13" s="65" t="str">
         <x:v>填写口播或对白全文</x:v>
       </x:c>
-      <x:c r="G13" s="40" t="str">
+      <x:c r="G13" s="65" t="str">
         <x:v>填写屏幕文字</x:v>
       </x:c>
-      <x:c r="H13" s="46" t="str">
+      <x:c r="H13" s="68" t="str">
         <x:v>填写一次生成可直接复制的完整提示词</x:v>
       </x:c>
-      <x:c r="I13" s="40" t="str">
+      <x:c r="I13" s="65" t="str">
         <x:v>填写与前后片段的衔接</x:v>
       </x:c>
-      <x:c r="J13" s="50" t="str">
+      <x:c r="J13" s="72" t="str">
         <x:v>填写需核对的画面与动作要点</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="142" customHeight="1">
-      <x:c r="A14" s="51" t="str">
+    <x:row r="14" ht="158" customHeight="1">
+      <x:c r="A14" s="32" t="str">
         <x:v>片段 04</x:v>
       </x:c>
-      <x:c r="B14" s="41" t="str">
+      <x:c r="B14" s="26" t="str">
         <x:v>填写整片位置、时长与画幅</x:v>
       </x:c>
-      <x:c r="C14" s="41" t="str">
+      <x:c r="C14" s="26" t="str">
         <x:v>填写关联分镜编号与段内节奏
 不要拆成独立生成任务</x:v>
       </x:c>
-      <x:c r="D14" s="41" t="str">
+      <x:c r="D14" s="26" t="str">
         <x:v>填写场景、构图、人物与动作</x:v>
       </x:c>
-      <x:c r="E14" s="44" t="str">
-        <x:v>在此嵌入实际参考图
-注明人物 / 产品 / 场景用途</x:v>
-      </x:c>
-      <x:c r="F14" s="41" t="str">
+      <x:c r="E14" s="27" t="str">
+        <x:v>填写本段图序与图 ID
+如图 1：P__ 产品参考
+图 2：R__ 角色参考
+图 3：S__ 场景参考
+按需增减，并嵌入对应真图</x:v>
+      </x:c>
+      <x:c r="F14" s="26" t="str">
         <x:v>填写口播或对白全文</x:v>
       </x:c>
-      <x:c r="G14" s="41" t="str">
+      <x:c r="G14" s="26" t="str">
         <x:v>填写屏幕文字</x:v>
       </x:c>
-      <x:c r="H14" s="46" t="str">
+      <x:c r="H14" s="68" t="str">
         <x:v>填写一次生成可直接复制的完整提示词</x:v>
       </x:c>
-      <x:c r="I14" s="41" t="str">
+      <x:c r="I14" s="26" t="str">
         <x:v>填写与前后片段的衔接</x:v>
       </x:c>
-      <x:c r="J14" s="52" t="str">
+      <x:c r="J14" s="29" t="str">
         <x:v>填写需核对的画面与动作要点</x:v>
       </x:c>
     </x:row>
@@ -899,4 +979,282 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFA8693B"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8.75" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.5" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.75" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17.5" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>参考资产</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="4" t="str">
+        <x:v>图编号是方案内部标识。图片嵌入表格供查看；生成时仍需上传所用实图，并按片段图序与用途关联。</x:v>
+      </x:c>
+      <x:c r="B2" s="4"/>
+      <x:c r="C2" s="4"/>
+      <x:c r="D2" s="4"/>
+      <x:c r="E2" s="4"/>
+      <x:c r="F2" s="4"/>
+      <x:c r="G2" s="4"/>
+      <x:c r="H2" s="4"/>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="7" t="str">
+        <x:v>资产清单</x:v>
+      </x:c>
+      <x:c r="B4" s="7"/>
+      <x:c r="C4" s="7"/>
+      <x:c r="D4" s="7"/>
+      <x:c r="E4" s="7"/>
+      <x:c r="F4" s="7"/>
+      <x:c r="G4" s="7"/>
+      <x:c r="H4" s="7"/>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="13" t="str">
+        <x:v>图 ID</x:v>
+      </x:c>
+      <x:c r="B5" s="13" t="str">
+        <x:v>类型</x:v>
+      </x:c>
+      <x:c r="C5" s="13" t="str">
+        <x:v>主体 / 场景名称</x:v>
+      </x:c>
+      <x:c r="D5" s="13" t="str">
+        <x:v>角度 / 状态</x:v>
+      </x:c>
+      <x:c r="E5" s="13" t="str">
+        <x:v>实际图</x:v>
+      </x:c>
+      <x:c r="F5" s="13" t="str">
+        <x:v>设定与本图约束用途</x:v>
+      </x:c>
+      <x:c r="G5" s="13" t="str">
+        <x:v>图像准备提示词 / 已有来源</x:v>
+      </x:c>
+      <x:c r="H5" s="13" t="str">
+        <x:v>关联片段</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="86" customHeight="1">
+      <x:c r="A6" s="30" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>产品参考</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>产品主视设定（模板示意）</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>外形、材质、标志、主角度与关键细节</x:v>
+      </x:c>
+      <x:c r="E6" s="19" t="str">
+        <x:v>待嵌入实际产品图
+非已生成</x:v>
+      </x:c>
+      <x:c r="F6" s="17" t="str">
+        <x:v>锁定产品外观，供产品出镜的片段复用。</x:v>
+      </x:c>
+      <x:c r="G6" s="20" t="str">
+        <x:v>填写产品设定图的准备提示词，或填写已有来源。</x:v>
+      </x:c>
+      <x:c r="H6" s="22" t="str">
+        <x:v>片段 01；按需复用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="86" customHeight="1">
+      <x:c r="A7" s="31" t="str">
+        <x:v>R01</x:v>
+      </x:c>
+      <x:c r="B7" s="18" t="str">
+        <x:v>角色参考</x:v>
+      </x:c>
+      <x:c r="C7" s="18" t="str">
+        <x:v>主角色身份与造型（模板示意）</x:v>
+      </x:c>
+      <x:c r="D7" s="18" t="str">
+        <x:v>可为真人、动漫或拟人角色；正面或三分之四视角</x:v>
+      </x:c>
+      <x:c r="E7" s="19" t="str">
+        <x:v>待嵌入实际角色图
+非已生成</x:v>
+      </x:c>
+      <x:c r="F7" s="18" t="str">
+        <x:v>锁定角色身份、造型、服装与辨识特征。</x:v>
+      </x:c>
+      <x:c r="G7" s="20" t="str">
+        <x:v>填写角色设定图的准备提示词，或填写已有来源。</x:v>
+      </x:c>
+      <x:c r="H7" s="24" t="str">
+        <x:v>片段 01；可跨片段复用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="86" customHeight="1">
+      <x:c r="A8" s="30" t="str">
+        <x:v>S01</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>场景参考</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>主场景设定（模板示意）</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>整体布局、主光方向、陈设与空间层次</x:v>
+      </x:c>
+      <x:c r="E8" s="19" t="str">
+        <x:v>待嵌入实际场景图
+非已生成</x:v>
+      </x:c>
+      <x:c r="F8" s="17" t="str">
+        <x:v>锁定场景结构、光线与陈设关系。</x:v>
+      </x:c>
+      <x:c r="G8" s="20" t="str">
+        <x:v>填写场景设定图的准备提示词，或填写已有来源。</x:v>
+      </x:c>
+      <x:c r="H8" s="22" t="str">
+        <x:v>片段 01；可跨片段复用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="76" customHeight="1">
+      <x:c r="A9" s="31" t="str">
+        <x:v>P02</x:v>
+      </x:c>
+      <x:c r="B9" s="18" t="str">
+        <x:v>可选产品细节</x:v>
+      </x:c>
+      <x:c r="C9" s="18" t="str">
+        <x:v>局部细节 / 另一产品角度</x:v>
+      </x:c>
+      <x:c r="D9" s="18" t="str">
+        <x:v>手持视角、材质细节或动作所需角度</x:v>
+      </x:c>
+      <x:c r="E9" s="19" t="str">
+        <x:v>按需嵌入实际图
+非已生成</x:v>
+      </x:c>
+      <x:c r="F9" s="18" t="str">
+        <x:v>仅在主图无法覆盖细节或特写时补充。</x:v>
+      </x:c>
+      <x:c r="G9" s="20" t="str">
+        <x:v>填写补充图准备提示词，或填写已有来源。</x:v>
+      </x:c>
+      <x:c r="H9" s="24" t="str">
+        <x:v>按需填写</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="76" customHeight="1">
+      <x:c r="A10" s="30" t="str">
+        <x:v>R02</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>可选角色视角</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>同一角色的另一视角</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="str">
+        <x:v>侧面、全身或动作起始姿态</x:v>
+      </x:c>
+      <x:c r="E10" s="19" t="str">
+        <x:v>按需嵌入实际图
+非已生成</x:v>
+      </x:c>
+      <x:c r="F10" s="17" t="str">
+        <x:v>仅在 R01 无法支撑动作连续性时补充。</x:v>
+      </x:c>
+      <x:c r="G10" s="20" t="str">
+        <x:v>填写补充图准备提示词，或填写已有来源。</x:v>
+      </x:c>
+      <x:c r="H10" s="22" t="str">
+        <x:v>按需填写</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="76" customHeight="1">
+      <x:c r="A11" s="31" t="str">
+        <x:v>S02</x:v>
+      </x:c>
+      <x:c r="B11" s="18" t="str">
+        <x:v>可选另一场景</x:v>
+      </x:c>
+      <x:c r="C11" s="18" t="str">
+        <x:v>另一场景设定</x:v>
+      </x:c>
+      <x:c r="D11" s="18" t="str">
+        <x:v>不同布局、光线或陈设关系</x:v>
+      </x:c>
+      <x:c r="E11" s="19" t="str">
+        <x:v>按需嵌入实际图
+非已生成</x:v>
+      </x:c>
+      <x:c r="F11" s="18" t="str">
+        <x:v>仅在片段切换到另一场景时补充。</x:v>
+      </x:c>
+      <x:c r="G11" s="20" t="str">
+        <x:v>填写补充图准备提示词，或填写已有来源。</x:v>
+      </x:c>
+      <x:c r="H11" s="24" t="str">
+        <x:v>按需填写</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="76" customHeight="1">
+      <x:c r="A12" s="32" t="str">
+        <x:v>C01</x:v>
+      </x:c>
+      <x:c r="B12" s="26" t="str">
+        <x:v>可选互动构图</x:v>
+      </x:c>
+      <x:c r="C12" s="26" t="str">
+        <x:v>互动起始构图</x:v>
+      </x:c>
+      <x:c r="D12" s="26" t="str">
+        <x:v>角色、产品与场景的相对位置和起始动作</x:v>
+      </x:c>
+      <x:c r="E12" s="27" t="str">
+        <x:v>按需嵌入实际图
+非已生成</x:v>
+      </x:c>
+      <x:c r="F12" s="26" t="str">
+        <x:v>仅在关键互动难以由单一设定图说明时补充。</x:v>
+      </x:c>
+      <x:c r="G12" s="28" t="str">
+        <x:v>填写构图指导提示词，或填写已有来源。</x:v>
+      </x:c>
+      <x:c r="H12" s="29" t="str">
+        <x:v>按需填写</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A4:H4"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>